<commit_message>
update testplan sequence again
</commit_message>
<xml_diff>
--- a/data/ROSA/test_item_sequence_all_cases.xlsx
+++ b/data/ROSA/test_item_sequence_all_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WTK_TestPlaner\data\ROSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA6989D-D089-4A7F-9889-4E20C2554777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B68194E-0186-40DF-9CD6-D26A94E433EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="25" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="18" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Case_01" sheetId="1" r:id="rId1"/>
@@ -3776,9 +3776,9 @@
   <dimension ref="A1:AY4"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="17.125" customWidth="1"/>
-    <col min="3" max="3" width="16.125" customWidth="1"/>
+    <col min="1" max="1" width="24.25" customWidth="1"/>
+    <col min="2" max="2" width="32.875" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
     <col min="5" max="5" width="14.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3951,34 +3951,37 @@
       <c r="A4" t="s">
         <v>53</v>
       </c>
-      <c r="B4" t="s">
-        <v>74</v>
+      <c r="B4">
+        <v>1</v>
       </c>
       <c r="C4" t="s">
         <v>74</v>
       </c>
       <c r="D4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" t="s">
         <v>75</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>74</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>66</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>67</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>68</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>69</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>70</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>70</v>
       </c>
     </row>

</xml_diff>